<commit_message>
add README, gitignore e alocacao original na planilha de resultados
- README.md: documenta nomenclatura das instancias (p, warm start, limites),
  modelos M1/M2/heuristica e significado de cada coluna da planilha
- .gitignore: exclui arquivos de dados sensiveis (rotas, Beneficiarios, Mananciais)
- adicionar_alocacao_original.py: calcula custo da alocacao original usando
  mapeamento exato GCDA->id_fonte via Mananciais_RN.csv
- resumo_custos.xlsx: coluna 'Custo Alocacao Original' + 7 gaps reestruturados
  (1 para confirmar M1A=M1D, 3 vs M1 Diario, 3 entre M2/Heuristica/Original)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/alocacao/saidas_3/resumo_custos.xlsx
+++ b/alocacao/saidas_3/resumo_custos.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -428,11 +428,16 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="34" customWidth="1" min="11" max="11"/>
-    <col width="92" customWidth="1" min="12" max="12"/>
-    <col width="97" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="92" customWidth="1" min="10" max="10"/>
+    <col width="97" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
+    <col width="27" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="33" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -478,27 +483,52 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Custo Alocação Original</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Caminho da Entrada</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Pasta de Saída</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Gap M1 Anual vs M1 Diário (%)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Gap M2 vs M1 Diário (%)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Gap Heurística vs M1 Diário (%)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Caminho da Entrada</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>Pasta de Saída</t>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Gap Original vs M1 Diário (%)</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Gap Heurística vs M2 (%)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Gap Original vs M2 (%)</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Gap Original vs Heurística (%)</t>
         </is>
       </c>
     </row>
@@ -531,24 +561,39 @@
       <c r="H2" s="3" t="n">
         <v>1861441.38</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="3" t="n">
+        <v>2845284.6</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00.csv</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_00</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>5.96</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="N2" s="4" t="n">
         <v>12.68</v>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00.csv</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_00</t>
-        </is>
+      <c r="O2" s="4" t="n">
+        <v>72.23999999999999</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>6.34</v>
+      </c>
+      <c r="Q2" s="4" t="n">
+        <v>62.55</v>
+      </c>
+      <c r="R2" s="4" t="n">
+        <v>52.85</v>
       </c>
     </row>
     <row r="3">
@@ -580,24 +625,39 @@
       <c r="H3" s="3" t="n">
         <v>1745834.52</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="I3" s="3" t="n">
+        <v>2880655.16</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00_350.csv</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_00_350</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>2.37</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="N3" s="4" t="n">
         <v>6.99</v>
       </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\00_350.csv</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_00_350</t>
-        </is>
+      <c r="O3" s="4" t="n">
+        <v>76.53</v>
+      </c>
+      <c r="P3" s="4" t="n">
+        <v>4.52</v>
+      </c>
+      <c r="Q3" s="4" t="n">
+        <v>72.45</v>
+      </c>
+      <c r="R3" s="4" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="4">
@@ -629,24 +689,39 @@
       <c r="H4" s="3" t="n">
         <v>1875173.57</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="3" t="n">
+        <v>3128657.42</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_01w24</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>1.67</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="N4" s="4" t="n">
         <v>5.95</v>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\01w24.csv</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_01w24</t>
-        </is>
+      <c r="O4" s="4" t="n">
+        <v>76.77</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>4.21</v>
+      </c>
+      <c r="Q4" s="4" t="n">
+        <v>73.86</v>
+      </c>
+      <c r="R4" s="4" t="n">
+        <v>66.84999999999999</v>
       </c>
     </row>
     <row r="5">
@@ -678,24 +753,39 @@
       <c r="H5" s="3" t="n">
         <v>1700765.66</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="3" t="n">
+        <v>2853346.85</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_10wLim</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>1.6</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="N5" s="4" t="n">
         <v>5.74</v>
       </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\10wLim.csv</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_10wLim</t>
-        </is>
+      <c r="O5" s="4" t="n">
+        <v>77.40000000000001</v>
+      </c>
+      <c r="P5" s="4" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>67.77</v>
       </c>
     </row>
     <row r="6">
@@ -727,24 +817,39 @@
       <c r="H6" s="3" t="n">
         <v>1789511.2</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I6" s="3" t="n">
+        <v>2992379.09</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_5072h</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>1.5</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="N6" s="4" t="n">
         <v>5.76</v>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\5072h.csv</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_5072h</t>
-        </is>
+      <c r="O6" s="4" t="n">
+        <v>76.86</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>74.23999999999999</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>67.22</v>
       </c>
     </row>
     <row r="7">
@@ -776,24 +881,39 @@
       <c r="H7" s="3" t="n">
         <v>1842701.13</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="3" t="n">
+        <v>3082478.25</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_50wLim</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>1.51</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="N7" s="4" t="n">
         <v>5.73</v>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\50wLim.csv</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_50wLim</t>
-        </is>
+      <c r="O7" s="4" t="n">
+        <v>76.87</v>
+      </c>
+      <c r="P7" s="4" t="n">
+        <v>4.15</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>74.23</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>67.28</v>
       </c>
     </row>
     <row r="8">
@@ -825,24 +945,39 @@
       <c r="H8" s="3" t="n">
         <v>1950294.03</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="3" t="n">
+        <v>3241210.02</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_75w00</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>1.76</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="N8" s="4" t="n">
         <v>6.35</v>
       </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\75w00.csv</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_75w00</t>
-        </is>
+      <c r="O8" s="4" t="n">
+        <v>76.73999999999999</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>4.51</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>73.69</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>66.19</v>
       </c>
     </row>
     <row r="9">
@@ -874,24 +1009,39 @@
       <c r="H9" s="3" t="n">
         <v>1950981.76</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="I9" s="3" t="n">
+        <v>2879167.06</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_heu_full</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>7.69</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="N9" s="4" t="n">
         <v>16.22</v>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_full.csv</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_heu_full</t>
-        </is>
+      <c r="O9" s="4" t="n">
+        <v>71.52</v>
+      </c>
+      <c r="P9" s="4" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>47.58</v>
       </c>
     </row>
     <row r="10">
@@ -923,24 +1073,39 @@
       <c r="H10" s="3" t="n">
         <v>1920901.5</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="I10" s="3" t="n">
+        <v>2849452.04</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_lim.csv</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_heu_lim</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>7.88</v>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="N10" s="4" t="n">
         <v>16.19</v>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\entradas\heu_lim.csv</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_3\alocacao_heu_lim</t>
-        </is>
+      <c r="O10" s="4" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>7.7</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>59.77</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>48.34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>